<commit_message>
fix: resolve data persistence issues and restore milestones from Drive
</commit_message>
<xml_diff>
--- a/data/tasks.xlsx
+++ b/data/tasks.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -619,7 +619,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Truck Unloading Project</t>
+          <t>R&amp;D Project</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -705,7 +705,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Truck Unloading Project</t>
+          <t>R&amp;D Project</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -766,7 +766,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Truck Unloading Project</t>
+          <t>R&amp;D Project</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -840,7 +840,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Truck Unloading Project</t>
+          <t>R&amp;D Project</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -909,7 +909,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Truck Unloading Project</t>
+          <t>R&amp;D Project</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -971,7 +971,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>Truck Unloading Project</t>
+          <t>R&amp;D Project</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -1029,7 +1029,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Truck Unloading Project</t>
+          <t>R&amp;D Project</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -1087,7 +1087,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>Truck Unloading Project</t>
+          <t>R&amp;D Project</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -1150,7 +1150,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>Truck Unloading Project</t>
+          <t>R&amp;D Project</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -1210,7 +1210,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>Truck Unloading Project</t>
+          <t>R&amp;D Project</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">

</xml_diff>

<commit_message>
revert: rollback to Wednesday state (ee0b887) as requested
</commit_message>
<xml_diff>
--- a/data/tasks.xlsx
+++ b/data/tasks.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -619,7 +619,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>R&amp;D Project</t>
+          <t>Truck Unloading Project</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -705,7 +705,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>R&amp;D Project</t>
+          <t>Truck Unloading Project</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -766,7 +766,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>R&amp;D Project</t>
+          <t>Truck Unloading Project</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -840,7 +840,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>R&amp;D Project</t>
+          <t>Truck Unloading Project</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -909,7 +909,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>R&amp;D Project</t>
+          <t>Truck Unloading Project</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -971,7 +971,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>R&amp;D Project</t>
+          <t>Truck Unloading Project</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -1029,7 +1029,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>R&amp;D Project</t>
+          <t>Truck Unloading Project</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -1087,7 +1087,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>R&amp;D Project</t>
+          <t>Truck Unloading Project</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -1150,7 +1150,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>R&amp;D Project</t>
+          <t>Truck Unloading Project</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -1210,7 +1210,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>R&amp;D Project</t>
+          <t>Truck Unloading Project</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">

</xml_diff>

<commit_message>
Fix Streamlit app restore and latest Drive sync
</commit_message>
<xml_diff>
--- a/data/tasks.xlsx
+++ b/data/tasks.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,16 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +34,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -45,21 +42,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -425,71 +413,71 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M12"/>
+  <dimension ref="A1:M13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Topic</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Task Name</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Start Date</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>End Date</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Completion %</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Hidden</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Project</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Employee</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Week</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Milestone_Text</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>Milestone_Author_Name</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>Milestone_Role</t>
         </is>
@@ -1233,6 +1221,67 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Dashboard</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Dataset collection and process</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>2026-04-27</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>2026-05-30</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>1</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="G13" t="b">
+        <v>0</v>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Truck Unloading Project</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Unassigned</t>
+        </is>
+      </c>
+      <c r="J13" t="n">
+        <v>17</v>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>Administrator</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>Admin</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>